<commit_message>
:bug: Fix repeat merge validation to respect dataframe_shift setting
When dataframe_shift is enabled, merged regions below dataframe anchors
are shifted out of the way. The post-shift validator was incorrectly
rejecting these shifted merges by checking overlap against the full
dataframe output range.

Fix:
- Pass dataframe_shift parameter to _validate_repeat_merges_do_not_overlap_dataframes
- When dataframe_shift='none', validate against full output range (strict)
- When dataframe_shift is enabled, validate only anchor cell (lenient)

This allows the playground template to compile successfully while still
catching genuine merge/dataframe conflicts when shifting is disabled.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/dataframe_shift/template.xlsx
+++ b/examples/dataframe_shift/template.xlsx
@@ -1,44 +1,82 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\06_Project_Dataport\mindoff-data-export\examples\dataframe_shift\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7310"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shift Demo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Shift Demo" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Repeat dataframe_shift repro</t>
+  </si>
+  <si>
+    <t>{{reports:repeat-start}}</t>
+  </si>
+  <si>
+    <t>Customer: {{customer_name:string}}</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>{{region:string}}</t>
+  </si>
+  <si>
+    <t>{{line_items_top:dataframe-content}}</t>
+  </si>
+  <si>
+    <t>{{between_label:string}}</t>
+  </si>
+  <si>
+    <t>{{line_items_bottom:dataframe-content}}</t>
+  </si>
+  <si>
+    <t>{{footer:string}}</t>
+  </si>
+  <si>
+    <t>{{reports:repeat-end}}</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <sz val="14"/>
+      <b/>
+      <sz val="13"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -50,11 +88,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFDE9D9"/>
+        <fgColor rgb="FFE8F4E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F1D3"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -62,90 +105,152 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="15">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -433,96 +538,94 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>dataframe_shift with repeat blocks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>{{reports:repeat-start}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Customer: {{customer_name:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{{region:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>{{line_items:dataframe-header}}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>{{note:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>{{line_items:dataframe-content}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>{{footer:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>{{reports:repeat-end}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Static footer after repeats</t>
-        </is>
-      </c>
+    <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+    </row>
+    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+    </row>
+    <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A6:D6"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="B4:D4"/>
   </mergeCells>

</xml_diff>

<commit_message>
🚀 Enhance dataframe shift handling and validation for merges (#15)
</commit_message>
<xml_diff>
--- a/examples/dataframe_shift/template.xlsx
+++ b/examples/dataframe_shift/template.xlsx
@@ -1,44 +1,82 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\06_Project_Dataport\mindoff-data-export\examples\dataframe_shift\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7310"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shift Demo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Shift Demo" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Repeat dataframe_shift repro</t>
+  </si>
+  <si>
+    <t>{{reports:repeat-start}}</t>
+  </si>
+  <si>
+    <t>Customer: {{customer_name:string}}</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>{{region:string}}</t>
+  </si>
+  <si>
+    <t>{{line_items_top:dataframe-content}}</t>
+  </si>
+  <si>
+    <t>{{between_label:string}}</t>
+  </si>
+  <si>
+    <t>{{line_items_bottom:dataframe-content}}</t>
+  </si>
+  <si>
+    <t>{{footer:string}}</t>
+  </si>
+  <si>
+    <t>{{reports:repeat-end}}</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <sz val="14"/>
+      <b/>
+      <sz val="13"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -50,11 +88,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFDE9D9"/>
+        <fgColor rgb="FFE8F4E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F1D3"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -62,90 +105,152 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="15">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -433,96 +538,94 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>dataframe_shift with repeat blocks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>{{reports:repeat-start}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Customer: {{customer_name:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Region</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{{region:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>{{line_items:dataframe-header}}</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>{{note:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>{{line_items:dataframe-content}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>{{footer:string}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>{{reports:repeat-end}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Static footer after repeats</t>
-        </is>
-      </c>
+    <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+    </row>
+    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="1:4" ht="32" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+    </row>
+    <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A6:D6"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="B4:D4"/>
   </mergeCells>

</xml_diff>